<commit_message>
Introduced Master Service and job Service to handle the API request.
all tests classes have been refactored to service classes
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tulinag/eclipse-workspace/PhoenixTestAutomationFramework/src/test/resources/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A3346F-BD3A-A94D-A786-3B13C2232BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BBACE6-38A3-BF4F-8B66-8346BC9C29AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33500" windowHeight="21100" activeTab="1" xr2:uid="{B7643BA3-8AA4-E84C-AEE3-A7B3D9579004}"/>
   </bookViews>
@@ -164,13 +164,13 @@
     <t>Schmidt</t>
   </si>
   <si>
-    <t>39556938683600</t>
-  </si>
-  <si>
-    <t>29526938683600</t>
-  </si>
-  <si>
     <t>464-509-3989</t>
+  </si>
+  <si>
+    <t>39556938683655</t>
+  </si>
+  <si>
+    <t>29526938683677</t>
   </si>
 </sst>
 </file>
@@ -1240,7 +1240,7 @@
         <v>34</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="V2" s="2" t="s">
         <v>35</v>
@@ -1276,13 +1276,13 @@
         <v>43</v>
       </c>
       <c r="AG2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AH2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AI2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AJ2" t="s">
         <v>43</v>
@@ -1336,7 +1336,7 @@
         <v>34</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="V3" s="2" t="s">
         <v>35</v>
@@ -1372,13 +1372,13 @@
         <v>43</v>
       </c>
       <c r="AG3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AH3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AI3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AJ3" t="s">
         <v>43</v>

</xml_diff>